<commit_message>
UPDATE : Menambahkan langkah-langkah untuk memilih warna pada format sel di file note.md dan memperbarui file latihan-excel-byGPT-04.xlsx
</commit_message>
<xml_diff>
--- a/belajar-excel-dasar/latihan-excel-dasar-byGPT/latihan-excel-byGPT-04.xlsx
+++ b/belajar-excel-dasar/latihan-excel-dasar-byGPT/latihan-excel-byGPT-04.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonovo\OneDrive\ドキュメント\belajar-excel\belajar-excel-dasar\latihan-excel-dasar-byGPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DC3B559-F306-4D0F-B2C9-9725C5B9233B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AEA49D-DEBA-4523-A4AE-81FECD2C21C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3CF9A7EE-0486-4030-98D4-2665C328FF1D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="pertemuan-byGPT-04" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>Hasil Ujian Akhir
 Mahasiswa Teknik Informatika</t>
@@ -49,24 +49,6 @@
     <t>Nilai</t>
   </si>
   <si>
-    <t>Andi</t>
-  </si>
-  <si>
-    <t>Budi</t>
-  </si>
-  <si>
-    <t>Citra</t>
-  </si>
-  <si>
-    <t>Diandra</t>
-  </si>
-  <si>
-    <t>Eko</t>
-  </si>
-  <si>
-    <t>Fitri</t>
-  </si>
-  <si>
     <t>Laki-laki</t>
   </si>
   <si>
@@ -74,13 +56,76 @@
   </si>
   <si>
     <t>IV</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t>Hasil</t>
+  </si>
+  <si>
+    <t>Total Nilai</t>
+  </si>
+  <si>
+    <t>Rata-rata Nilai</t>
+  </si>
+  <si>
+    <t>Nilai Tertinggi</t>
+  </si>
+  <si>
+    <t>Nilai Terendah</t>
+  </si>
+  <si>
+    <t>Jumlah Mahasiswa</t>
+  </si>
+  <si>
+    <t>Andry Hakim</t>
+  </si>
+  <si>
+    <t>Budi Cahyo</t>
+  </si>
+  <si>
+    <t>Citra Lestari</t>
+  </si>
+  <si>
+    <t>Diandra Zahra</t>
+  </si>
+  <si>
+    <t>Eko Kurniawan Khanedy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fitriani </t>
+  </si>
+  <si>
+    <t>Jumlah Data Terisi (Kolom Nama)</t>
+  </si>
+  <si>
+    <t>RUMUS</t>
+  </si>
+  <si>
+    <t>SUM</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>MIN</t>
+  </si>
+  <si>
+    <t>COUNT</t>
+  </si>
+  <si>
+    <t>COUNTA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,8 +151,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -126,8 +178,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -150,16 +214,123 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -168,12 +339,101 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -491,10 +751,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97AED4A9-A615-4532-A398-050F2E07AC3E}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -502,159 +763,254 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="13" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="10">
+        <v>12101001</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="1">
-        <v>12101001</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3">
-        <v>90</v>
+      <c r="E4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="14">
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1">
         <v>12101002</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="3">
-        <v>87</v>
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="7">
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1">
         <v>12101003</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="3">
-        <v>96</v>
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="7">
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C7" s="1">
         <v>12101004</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="3">
-        <v>84</v>
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="7">
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C8" s="1">
         <v>12101005</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="3">
-        <v>76</v>
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="7">
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C9" s="1">
         <v>12101006</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="7">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="17">
+        <f>SUM(F4:F9)</f>
+        <v>507</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="18">
+        <f>AVERAGE(F4:F9)</f>
+        <v>84.5</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="B15" s="18">
+        <f>MAX(F4:F9)</f>
+        <v>95</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="3">
-        <v>80</v>
+      <c r="B16" s="18">
+        <f>MIN(F4:F9)</f>
+        <v>56</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="18">
+        <f>COUNT(A4:A9)</f>
+        <v>6</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="19">
+        <f>COUNTA(B4:B9)</f>
+        <v>6</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A4:F9">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="A4:F9 B12">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A13:B17 A18">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13:C18">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>